<commit_message>
update Unit Test Design
</commit_message>
<xml_diff>
--- a/Testing/TestPlan_Group06.xlsx
+++ b/Testing/TestPlan_Group06.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="878" uniqueCount="508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="557">
   <si>
     <t/>
   </si>
@@ -743,6 +743,72 @@
     <t>Test Email</t>
   </si>
   <si>
+    <t>UT071</t>
+  </si>
+  <si>
+    <t>Missing requirement of 'username', 'password'  from user information</t>
+  </si>
+  <si>
+    <t>UT072</t>
+  </si>
+  <si>
+    <t>Missing requirement of 'username' , 'email' from user information</t>
+  </si>
+  <si>
+    <t>UT073</t>
+  </si>
+  <si>
+    <t>Missing requirement of 'email', 'password'  from user information</t>
+  </si>
+  <si>
+    <t>UT074</t>
+  </si>
+  <si>
+    <t>Missing requirements of all three fields from user information</t>
+  </si>
+  <si>
+    <t>UT075</t>
+  </si>
+  <si>
+    <t>Missing requirement of 'email'  from delivery information</t>
+  </si>
+  <si>
+    <t>UT076</t>
+  </si>
+  <si>
+    <t>Missing requirement of 'phoneNumber'  from delivery information</t>
+  </si>
+  <si>
+    <t>UT077</t>
+  </si>
+  <si>
+    <t>No missing requirement from delivery information</t>
+  </si>
+  <si>
+    <t>UT078</t>
+  </si>
+  <si>
+    <t>Missing requirements of all two fields from delivery information</t>
+  </si>
+  <si>
+    <t>UT079</t>
+  </si>
+  <si>
+    <t>Test on 'checkEligibilityForRushDeliveryOfCartItems' method</t>
+  </si>
+  <si>
+    <t>UT080</t>
+  </si>
+  <si>
+    <t>Test case TRUE on 'checkIfUsernameAlreadyExists' method</t>
+  </si>
+  <si>
+    <t>UT081</t>
+  </si>
+  <si>
+    <t>Test case FALSE on 'checkIfUsernameAlreadyExists' method</t>
+  </si>
+  <si>
     <t>4.2. Test Suite for UC001-"View Product Details"</t>
   </si>
   <si>
@@ -866,7 +932,7 @@
     <t>UT056, UT057, UT058, UT059, UT060</t>
   </si>
   <si>
-    <t>4.. Test Suite for UC00-"Place Order"</t>
+    <t>4.8. Test Suite for UC00-"Place Order"</t>
   </si>
   <si>
     <t>Place Order Test Suite</t>
@@ -878,10 +944,43 @@
     <t>UT061 - UT070</t>
   </si>
   <si>
-    <t>4.8. Test Suite for UC "Create New User"</t>
+    <t>4.9. Test Suite for UC008 "Manage User"</t>
   </si>
   <si>
-    <t>4.9. Test Suite for UC "Update User Information"</t>
+    <t>User Controller Test Suite</t>
+  </si>
+  <si>
+    <t>Tests the functionality for input verification and event handlers when managing users</t>
+  </si>
+  <si>
+    <t>UT052, UT053, UT054, UT055, UT071, UT072, UT073, UT074</t>
+  </si>
+  <si>
+    <t>User Service Test Suite</t>
+  </si>
+  <si>
+    <t>Tests the functionality for data retrival and processings with related 'User' data</t>
+  </si>
+  <si>
+    <t>UT080, UT081</t>
+  </si>
+  <si>
+    <t>4.9. Test Suite for UC007 "Place Rush Order"</t>
+  </si>
+  <si>
+    <t>Place Rush Controller Test Suite</t>
+  </si>
+  <si>
+    <t>Tests the functionality for input verification and event handlers when users decide to select rush delivery method</t>
+  </si>
+  <si>
+    <t>UT075, UT076, UT077, UT078</t>
+  </si>
+  <si>
+    <t>Cart Service Test Suite</t>
+  </si>
+  <si>
+    <t>Tests the functionality for checking condition for rush delivery of items from cart</t>
   </si>
   <si>
     <t>5. Test Case Details</t>
@@ -1448,9 +1547,6 @@
     <t>Bulk‐operation limit</t>
   </si>
   <si>
-    <t>s</t>
-  </si>
-  <si>
     <t>Clerk tries to approve without Manager role</t>
   </si>
   <si>
@@ -1709,6 +1805,71 @@
     <t>Notification test</t>
   </si>
   <si>
+    <t>user = new User("1, "bad user", "user@example.com", "nopass", "admin", true, LocalDateTime.now().minusDays(1), LocalDateTime.now())</t>
+  </si>
+  <si>
+    <t>user = new User("1, "bad!user", "bademail", "Strong1@pass", "admin", true, LocalDateTime.now().minusDays(1), LocalDateTime.now())</t>
+  </si>
+  <si>
+    <t>user = new User("1, "validUser", "bad@", "123", "admin", true, LocalDateTime.now().minusDays(1), LocalDateTime.now())</t>
+  </si>
+  <si>
+    <t>user = new User("1, "!", "noemail", "123", "admin", true, LocalDateTime.now().minusDays(1), LocalDateTime.now())</t>
+  </si>
+  <si>
+    <t>PlaceRushOrderController.checkIfDeliveryInfoMeetsPolicies(deliveryInfo: DeliveryInfo)</t>
+  </si>
+  <si>
+    <t>deliveryInfo = new DeliveryInfo(2, "Thomas", "@gmail.com", "0912345678", "Hanoi", "Ba Dinh")</t>
+  </si>
+  <si>
+    <t>deliveryInfo = new DeliveryInfo(3, "Thomas", "user@gmail.com", "0912378", "Thai Binh", "Dong Hung")</t>
+  </si>
+  <si>
+    <t>deliveryInfo = new DeliveryInfo(1, "John Doe", "user@example.com", "0912345678", "Hanoi", "Ba Dinh")</t>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>deliveryInfo = new DeliveryInfo(4, "Shelly", "</t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>shelly123gmail.com</t>
+    </r>
+    <r>
+      <rPr/>
+      <t>", "1234", "Hanoi", "Thanh Xuan")</t>
+    </r>
+  </si>
+  <si>
+    <t>Return Map&lt;Integer, Boolean&gt;, map cartItemID to TRUE if eligible, FALSE if not</t>
+  </si>
+  <si>
+    <t>CartService.checkEligibilityForRushDeliveryOfCartItems(cartItems: List&lt;CartItems&gt;</t>
+  </si>
+  <si>
+    <t>cartItems = Arrays.asList(new CartItem(101, 1, 1, 2, 120.0f), new CartItem(102, 2, 1, 5, 50.0f), new CartItem(103, 3, 1, 3, 75.0f))</t>
+  </si>
+  <si>
+    <t>new HashMap&lt;String, Integer&gt;() {{put(101, true);  put(102, false);  put(103, false);</t>
+  </si>
+  <si>
+    <t>Iterating through all 'User' instance to check existence of 'username'</t>
+  </si>
+  <si>
+    <t>UserService.checkIfUsernameAlreadyExists(username: String)</t>
+  </si>
+  <si>
+    <t>username = "alice123"</t>
+  </si>
+  <si>
+    <t>username = "thomas124"</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <rFont val="Calibri"/>
@@ -1813,7 +1974,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -1916,6 +2077,13 @@
     </font>
     <font>
       <b/>
+      <sz val="13.0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -1936,6 +2104,10 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="6">
@@ -2045,7 +2217,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="90">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2167,8 +2339,23 @@
     <xf borderId="4" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -2242,31 +2429,40 @@
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="5" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="7" fillId="5" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="22" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
@@ -62680,11 +62876,12 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="8.14"/>
+    <col customWidth="1" min="1" max="1" width="11.86"/>
     <col customWidth="1" min="2" max="2" width="50.14"/>
-    <col customWidth="1" min="3" max="6" width="8.86"/>
+    <col customWidth="1" min="3" max="6" width="10.86"/>
     <col customWidth="1" min="7" max="7" width="14.71"/>
-    <col customWidth="1" min="8" max="27" width="8.86"/>
+    <col customWidth="1" min="8" max="9" width="10.86"/>
+    <col customWidth="1" min="10" max="27" width="8.86"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -64154,421 +64351,697 @@
       <c r="I75" s="32"/>
     </row>
     <row r="76">
-      <c r="A76" s="26"/>
-      <c r="B76" s="45"/>
-      <c r="C76" s="26"/>
-      <c r="D76" s="30"/>
-      <c r="E76" s="32"/>
-      <c r="F76" s="30"/>
-      <c r="G76" s="30"/>
-      <c r="H76" s="30"/>
-      <c r="I76" s="30"/>
+      <c r="A76" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="B76" s="45" t="s">
+        <v>182</v>
+      </c>
+      <c r="C76" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D76" s="37"/>
+      <c r="E76" s="37"/>
+      <c r="F76" s="37"/>
+      <c r="G76" s="37"/>
+      <c r="H76" s="37"/>
+      <c r="I76" s="32" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="46" t="s">
-        <v>181</v>
-      </c>
+      <c r="A77" s="27" t="s">
+        <v>183</v>
+      </c>
+      <c r="B77" s="45" t="s">
+        <v>184</v>
+      </c>
+      <c r="C77" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D77" s="37"/>
+      <c r="E77" s="37"/>
+      <c r="F77" s="37"/>
+      <c r="G77" s="37"/>
+      <c r="H77" s="37"/>
+      <c r="I77" s="32"/>
     </row>
     <row r="78">
-      <c r="A78" s="47" t="s">
-        <v>182</v>
-      </c>
-      <c r="B78" s="47" t="s">
-        <v>183</v>
-      </c>
-      <c r="C78" s="48" t="s">
-        <v>184</v>
-      </c>
-      <c r="D78" s="22"/>
-      <c r="E78" s="23"/>
-      <c r="F78" s="48" t="s">
+      <c r="A78" s="27" t="s">
         <v>185</v>
       </c>
-      <c r="G78" s="23"/>
-      <c r="M78" s="31"/>
-      <c r="N78" s="31"/>
-      <c r="O78" s="31"/>
-      <c r="P78" s="31"/>
+      <c r="B78" s="45" t="s">
+        <v>186</v>
+      </c>
+      <c r="C78" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D78" s="37"/>
+      <c r="E78" s="37"/>
+      <c r="F78" s="37"/>
+      <c r="G78" s="37"/>
+      <c r="H78" s="37"/>
+      <c r="I78" s="32"/>
     </row>
     <row r="79">
-      <c r="A79" s="49" t="s">
-        <v>186</v>
-      </c>
-      <c r="B79" s="50" t="s">
+      <c r="A79" s="27" t="s">
         <v>187</v>
       </c>
-      <c r="C79" s="51" t="s">
+      <c r="B79" s="45" t="s">
         <v>188</v>
       </c>
-      <c r="D79" s="22"/>
-      <c r="E79" s="23"/>
-      <c r="F79" s="52" t="s">
+      <c r="C79" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D79" s="37"/>
+      <c r="E79" s="37"/>
+      <c r="F79" s="37"/>
+      <c r="G79" s="37"/>
+      <c r="H79" s="37"/>
+      <c r="I79" s="32"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="27" t="s">
         <v>189</v>
       </c>
-      <c r="G79" s="23"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="53"/>
-      <c r="B80" s="53"/>
-      <c r="C80" s="19"/>
-      <c r="D80" s="19"/>
-      <c r="E80" s="19"/>
-      <c r="F80" s="54"/>
-      <c r="G80" s="54"/>
-    </row>
-    <row r="81" ht="18.75" customHeight="1">
-      <c r="A81" s="53"/>
-      <c r="B81" s="53"/>
-      <c r="C81" s="19"/>
-      <c r="D81" s="19"/>
-      <c r="E81" s="19"/>
-      <c r="F81" s="54"/>
-      <c r="G81" s="54"/>
+      <c r="B80" s="45" t="s">
+        <v>190</v>
+      </c>
+      <c r="C80" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D80" s="37"/>
+      <c r="E80" s="37"/>
+      <c r="F80" s="37"/>
+      <c r="G80" s="37"/>
+      <c r="H80" s="37"/>
+      <c r="I80" s="32"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="27" t="s">
+        <v>191</v>
+      </c>
+      <c r="B81" s="45" t="s">
+        <v>192</v>
+      </c>
+      <c r="C81" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D81" s="37"/>
+      <c r="E81" s="37"/>
+      <c r="F81" s="37"/>
+      <c r="G81" s="37"/>
+      <c r="H81" s="37"/>
+      <c r="I81" s="32"/>
     </row>
     <row r="82">
-      <c r="A82" s="46" t="s">
-        <v>190</v>
-      </c>
+      <c r="A82" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="B82" s="45" t="s">
+        <v>194</v>
+      </c>
+      <c r="C82" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D82" s="37"/>
+      <c r="E82" s="37"/>
+      <c r="F82" s="37"/>
+      <c r="G82" s="37"/>
+      <c r="H82" s="37"/>
+      <c r="I82" s="32"/>
     </row>
     <row r="83">
-      <c r="A83" s="47" t="s">
-        <v>182</v>
-      </c>
-      <c r="B83" s="47" t="s">
-        <v>183</v>
-      </c>
-      <c r="C83" s="48" t="s">
-        <v>184</v>
-      </c>
-      <c r="D83" s="22"/>
-      <c r="E83" s="23"/>
-      <c r="F83" s="48" t="s">
-        <v>185</v>
-      </c>
-      <c r="G83" s="23"/>
+      <c r="A83" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="B83" s="45" t="s">
+        <v>196</v>
+      </c>
+      <c r="C83" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D83" s="37"/>
+      <c r="E83" s="37"/>
+      <c r="F83" s="37"/>
+      <c r="G83" s="37"/>
+      <c r="H83" s="37"/>
+      <c r="I83" s="32"/>
     </row>
     <row r="84">
-      <c r="A84" s="49" t="s">
-        <v>186</v>
-      </c>
-      <c r="B84" s="50" t="s">
-        <v>191</v>
-      </c>
-      <c r="C84" s="51" t="s">
-        <v>192</v>
-      </c>
-      <c r="D84" s="22"/>
-      <c r="E84" s="23"/>
-      <c r="F84" s="52" t="s">
-        <v>193</v>
-      </c>
-      <c r="G84" s="23"/>
-    </row>
-    <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="49" t="s">
-        <v>194</v>
-      </c>
-      <c r="B85" s="50" t="s">
-        <v>195</v>
-      </c>
-      <c r="C85" s="51" t="s">
-        <v>196</v>
-      </c>
-      <c r="D85" s="22"/>
-      <c r="E85" s="23"/>
-      <c r="F85" s="52" t="s">
+      <c r="A84" s="27" t="s">
         <v>197</v>
       </c>
-      <c r="G85" s="23"/>
-    </row>
-    <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="49" t="s">
+      <c r="B84" s="45" t="s">
         <v>198</v>
       </c>
-      <c r="B86" s="50" t="s">
+      <c r="C84" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D84" s="37"/>
+      <c r="E84" s="37"/>
+      <c r="F84" s="37"/>
+      <c r="G84" s="37"/>
+      <c r="H84" s="37"/>
+      <c r="I84" s="32"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="27" t="s">
         <v>199</v>
       </c>
-      <c r="C86" s="51" t="s">
+      <c r="B85" s="45" t="s">
         <v>200</v>
       </c>
-      <c r="D86" s="22"/>
-      <c r="E86" s="23"/>
-      <c r="F86" s="52" t="s">
+      <c r="C85" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D85" s="37"/>
+      <c r="E85" s="37"/>
+      <c r="F85" s="37"/>
+      <c r="G85" s="37"/>
+      <c r="H85" s="37"/>
+      <c r="I85" s="32"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="27" t="s">
         <v>201</v>
       </c>
-      <c r="G86" s="23"/>
-    </row>
-    <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="49" t="s">
+      <c r="B86" s="45" t="s">
         <v>202</v>
       </c>
-      <c r="B87" s="50" t="s">
+      <c r="C86" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="D86" s="37"/>
+      <c r="E86" s="37"/>
+      <c r="F86" s="37"/>
+      <c r="G86" s="37"/>
+      <c r="H86" s="37"/>
+      <c r="I86" s="32"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="46"/>
+      <c r="B87" s="47"/>
+      <c r="C87" s="48"/>
+      <c r="D87" s="49"/>
+      <c r="E87" s="50"/>
+      <c r="F87" s="49"/>
+      <c r="G87" s="49"/>
+      <c r="H87" s="49"/>
+      <c r="I87" s="49"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="51" t="s">
         <v>203</v>
       </c>
-      <c r="C87" s="51" t="s">
+    </row>
+    <row r="89">
+      <c r="A89" s="52" t="s">
         <v>204</v>
       </c>
-      <c r="D87" s="22"/>
-      <c r="E87" s="23"/>
-      <c r="F87" s="52" t="s">
+      <c r="B89" s="52" t="s">
         <v>205</v>
       </c>
-      <c r="G87" s="23"/>
-    </row>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" s="31"/>
-      <c r="B89" s="31"/>
-      <c r="C89" s="31"/>
-      <c r="D89" s="31"/>
-    </row>
-    <row r="90" ht="15.75" customHeight="1"/>
-    <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" s="46" t="s">
+      <c r="C89" s="53" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" s="47" t="s">
-        <v>182</v>
-      </c>
-      <c r="B92" s="47" t="s">
-        <v>183</v>
-      </c>
-      <c r="C92" s="48" t="s">
-        <v>184</v>
-      </c>
-      <c r="D92" s="22"/>
-      <c r="E92" s="23"/>
-      <c r="F92" s="48" t="s">
-        <v>185</v>
-      </c>
-      <c r="G92" s="23"/>
-    </row>
-    <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="49" t="s">
-        <v>186</v>
-      </c>
-      <c r="B93" s="50" t="s">
+      <c r="D89" s="22"/>
+      <c r="E89" s="23"/>
+      <c r="F89" s="53" t="s">
         <v>207</v>
       </c>
-      <c r="C93" s="51" t="s">
+      <c r="G89" s="23"/>
+      <c r="M89" s="31"/>
+      <c r="N89" s="31"/>
+      <c r="O89" s="31"/>
+      <c r="P89" s="31"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="54" t="s">
         <v>208</v>
       </c>
-      <c r="D93" s="22"/>
-      <c r="E93" s="23"/>
-      <c r="F93" s="52" t="s">
+      <c r="B90" s="55" t="s">
         <v>209</v>
       </c>
-      <c r="G93" s="23"/>
-    </row>
-    <row r="94" ht="15.75" customHeight="1">
-      <c r="A94" s="55" t="s">
+      <c r="C90" s="56" t="s">
         <v>210</v>
       </c>
-      <c r="C94" s="56"/>
-      <c r="D94" s="56"/>
-      <c r="E94" s="56"/>
-      <c r="F94" s="56"/>
-      <c r="G94" s="56"/>
-    </row>
-    <row r="95" ht="15.75" customHeight="1">
-      <c r="A95" s="57" t="s">
-        <v>182</v>
-      </c>
-      <c r="B95" s="58" t="s">
-        <v>183</v>
-      </c>
-      <c r="C95" s="59" t="s">
-        <v>184</v>
+      <c r="D90" s="22"/>
+      <c r="E90" s="23"/>
+      <c r="F90" s="57" t="s">
+        <v>211</v>
+      </c>
+      <c r="G90" s="23"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="58"/>
+      <c r="B91" s="58"/>
+      <c r="C91" s="19"/>
+      <c r="D91" s="19"/>
+      <c r="E91" s="19"/>
+      <c r="F91" s="59"/>
+      <c r="G91" s="59"/>
+    </row>
+    <row r="92" ht="18.75" customHeight="1">
+      <c r="A92" s="58"/>
+      <c r="B92" s="58"/>
+      <c r="C92" s="19"/>
+      <c r="D92" s="19"/>
+      <c r="E92" s="19"/>
+      <c r="F92" s="59"/>
+      <c r="G92" s="59"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="51" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="52" t="s">
+        <v>204</v>
+      </c>
+      <c r="B94" s="52" t="s">
+        <v>205</v>
+      </c>
+      <c r="C94" s="53" t="s">
+        <v>206</v>
+      </c>
+      <c r="D94" s="22"/>
+      <c r="E94" s="23"/>
+      <c r="F94" s="53" t="s">
+        <v>207</v>
+      </c>
+      <c r="G94" s="23"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="54" t="s">
+        <v>208</v>
+      </c>
+      <c r="B95" s="55" t="s">
+        <v>213</v>
+      </c>
+      <c r="C95" s="56" t="s">
+        <v>214</v>
       </c>
       <c r="D95" s="22"/>
       <c r="E95" s="23"/>
-      <c r="F95" s="59" t="s">
-        <v>185</v>
+      <c r="F95" s="57" t="s">
+        <v>215</v>
       </c>
       <c r="G95" s="23"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
-      <c r="A96" s="60" t="s">
-        <v>186</v>
-      </c>
-      <c r="B96" s="61" t="s">
-        <v>211</v>
-      </c>
-      <c r="C96" s="62" t="s">
-        <v>212</v>
+      <c r="A96" s="54" t="s">
+        <v>216</v>
+      </c>
+      <c r="B96" s="55" t="s">
+        <v>217</v>
+      </c>
+      <c r="C96" s="56" t="s">
+        <v>218</v>
       </c>
       <c r="D96" s="22"/>
       <c r="E96" s="23"/>
-      <c r="F96" s="62" t="s">
-        <v>213</v>
+      <c r="F96" s="57" t="s">
+        <v>219</v>
       </c>
       <c r="G96" s="23"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
-      <c r="A97" s="63" t="s">
-        <v>214</v>
-      </c>
-      <c r="C97" s="64"/>
-      <c r="D97" s="64"/>
-      <c r="E97" s="65"/>
-      <c r="F97" s="66"/>
-      <c r="G97" s="66"/>
+      <c r="A97" s="54" t="s">
+        <v>220</v>
+      </c>
+      <c r="B97" s="55" t="s">
+        <v>221</v>
+      </c>
+      <c r="C97" s="56" t="s">
+        <v>222</v>
+      </c>
+      <c r="D97" s="22"/>
+      <c r="E97" s="23"/>
+      <c r="F97" s="57" t="s">
+        <v>223</v>
+      </c>
+      <c r="G97" s="23"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
-      <c r="A98" s="57" t="s">
-        <v>182</v>
-      </c>
-      <c r="B98" s="58" t="s">
-        <v>183</v>
-      </c>
-      <c r="C98" s="59" t="s">
-        <v>184</v>
+      <c r="A98" s="54" t="s">
+        <v>224</v>
+      </c>
+      <c r="B98" s="55" t="s">
+        <v>225</v>
+      </c>
+      <c r="C98" s="56" t="s">
+        <v>226</v>
       </c>
       <c r="D98" s="22"/>
       <c r="E98" s="23"/>
-      <c r="F98" s="59" t="s">
-        <v>185</v>
+      <c r="F98" s="57" t="s">
+        <v>227</v>
       </c>
       <c r="G98" s="23"/>
     </row>
-    <row r="99" ht="15.75" customHeight="1">
-      <c r="A99" s="60" t="s">
-        <v>186</v>
-      </c>
-      <c r="B99" s="61" t="s">
-        <v>215</v>
-      </c>
-      <c r="C99" s="62" t="s">
-        <v>216</v>
-      </c>
-      <c r="D99" s="22"/>
-      <c r="E99" s="23"/>
-      <c r="F99" s="62" t="s">
-        <v>217</v>
-      </c>
-      <c r="G99" s="23"/>
-    </row>
-    <row r="100" ht="15.75" customHeight="1"/>
-    <row r="101" ht="15.75" customHeight="1">
-      <c r="A101" s="46" t="s">
-        <v>218</v>
-      </c>
-    </row>
+    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1">
+      <c r="A100" s="31"/>
+      <c r="B100" s="31"/>
+      <c r="C100" s="31"/>
+      <c r="D100" s="31"/>
+    </row>
+    <row r="101" ht="15.75" customHeight="1"/>
     <row r="102" ht="15.75" customHeight="1">
-      <c r="A102" s="47" t="s">
-        <v>182</v>
-      </c>
-      <c r="B102" s="47" t="s">
-        <v>183</v>
-      </c>
-      <c r="C102" s="48" t="s">
-        <v>184</v>
-      </c>
-      <c r="D102" s="22"/>
-      <c r="E102" s="23"/>
-      <c r="F102" s="48" t="s">
-        <v>185</v>
-      </c>
-      <c r="G102" s="23"/>
+      <c r="A102" s="51" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="103" ht="15.75" customHeight="1">
-      <c r="A103" s="49" t="s">
-        <v>186</v>
-      </c>
-      <c r="B103" s="50" t="s">
-        <v>219</v>
-      </c>
-      <c r="C103" s="51" t="s">
-        <v>220</v>
+      <c r="A103" s="52" t="s">
+        <v>204</v>
+      </c>
+      <c r="B103" s="52" t="s">
+        <v>205</v>
+      </c>
+      <c r="C103" s="53" t="s">
+        <v>206</v>
       </c>
       <c r="D103" s="22"/>
       <c r="E103" s="23"/>
-      <c r="F103" s="52" t="s">
-        <v>221</v>
+      <c r="F103" s="53" t="s">
+        <v>207</v>
       </c>
       <c r="G103" s="23"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
-      <c r="A104" s="53"/>
-      <c r="B104" s="67"/>
-      <c r="C104" s="68"/>
-      <c r="D104" s="68"/>
-      <c r="E104" s="68"/>
-      <c r="F104" s="69"/>
-      <c r="G104" s="69"/>
+      <c r="A104" s="54" t="s">
+        <v>208</v>
+      </c>
+      <c r="B104" s="55" t="s">
+        <v>229</v>
+      </c>
+      <c r="C104" s="56" t="s">
+        <v>230</v>
+      </c>
+      <c r="D104" s="22"/>
+      <c r="E104" s="23"/>
+      <c r="F104" s="57" t="s">
+        <v>231</v>
+      </c>
+      <c r="G104" s="23"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
-      <c r="A105" s="46" t="s">
-        <v>222</v>
-      </c>
+      <c r="A105" s="60" t="s">
+        <v>232</v>
+      </c>
+      <c r="C105" s="61"/>
+      <c r="D105" s="61"/>
+      <c r="E105" s="61"/>
+      <c r="F105" s="61"/>
+      <c r="G105" s="61"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
-      <c r="A106" s="47" t="s">
-        <v>182</v>
-      </c>
-      <c r="B106" s="47" t="s">
-        <v>183</v>
-      </c>
-      <c r="C106" s="48" t="s">
-        <v>184</v>
+      <c r="A106" s="62" t="s">
+        <v>204</v>
+      </c>
+      <c r="B106" s="63" t="s">
+        <v>205</v>
+      </c>
+      <c r="C106" s="64" t="s">
+        <v>206</v>
       </c>
       <c r="D106" s="22"/>
       <c r="E106" s="23"/>
-      <c r="F106" s="48" t="s">
-        <v>185</v>
+      <c r="F106" s="64" t="s">
+        <v>207</v>
       </c>
       <c r="G106" s="23"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
-      <c r="A107" s="49" t="s">
-        <v>186</v>
-      </c>
-      <c r="B107" s="50" t="s">
-        <v>223</v>
-      </c>
-      <c r="C107" s="51" t="s">
-        <v>224</v>
+      <c r="A107" s="65" t="s">
+        <v>208</v>
+      </c>
+      <c r="B107" s="66" t="s">
+        <v>233</v>
+      </c>
+      <c r="C107" s="67" t="s">
+        <v>234</v>
       </c>
       <c r="D107" s="22"/>
       <c r="E107" s="23"/>
-      <c r="F107" s="52" t="s">
-        <v>225</v>
+      <c r="F107" s="67" t="s">
+        <v>235</v>
       </c>
       <c r="G107" s="23"/>
     </row>
-    <row r="108" ht="15.75" customHeight="1"/>
-    <row r="109" ht="15.75" customHeight="1"/>
+    <row r="108" ht="15.75" customHeight="1">
+      <c r="A108" s="68" t="s">
+        <v>236</v>
+      </c>
+      <c r="C108" s="69"/>
+      <c r="D108" s="69"/>
+      <c r="E108" s="70"/>
+      <c r="F108" s="71"/>
+      <c r="G108" s="71"/>
+    </row>
+    <row r="109" ht="15.75" customHeight="1">
+      <c r="A109" s="62" t="s">
+        <v>204</v>
+      </c>
+      <c r="B109" s="63" t="s">
+        <v>205</v>
+      </c>
+      <c r="C109" s="64" t="s">
+        <v>206</v>
+      </c>
+      <c r="D109" s="22"/>
+      <c r="E109" s="23"/>
+      <c r="F109" s="64" t="s">
+        <v>207</v>
+      </c>
+      <c r="G109" s="23"/>
+    </row>
     <row r="110" ht="15.75" customHeight="1">
-      <c r="A110" s="1" t="s">
-        <v>226</v>
-      </c>
+      <c r="A110" s="65" t="s">
+        <v>208</v>
+      </c>
+      <c r="B110" s="66" t="s">
+        <v>237</v>
+      </c>
+      <c r="C110" s="67" t="s">
+        <v>238</v>
+      </c>
+      <c r="D110" s="22"/>
+      <c r="E110" s="23"/>
+      <c r="F110" s="67" t="s">
+        <v>239</v>
+      </c>
+      <c r="G110" s="23"/>
     </row>
     <row r="111" ht="15.75" customHeight="1"/>
-    <row r="112" ht="15.75" customHeight="1"/>
-    <row r="113" ht="15.75" customHeight="1"/>
-    <row r="114" ht="15.75" customHeight="1"/>
-    <row r="115" ht="15.75" customHeight="1"/>
+    <row r="112" ht="15.75" customHeight="1">
+      <c r="A112" s="51" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="113" ht="15.75" customHeight="1">
+      <c r="A113" s="52" t="s">
+        <v>204</v>
+      </c>
+      <c r="B113" s="52" t="s">
+        <v>205</v>
+      </c>
+      <c r="C113" s="53" t="s">
+        <v>206</v>
+      </c>
+      <c r="D113" s="22"/>
+      <c r="E113" s="23"/>
+      <c r="F113" s="53" t="s">
+        <v>207</v>
+      </c>
+      <c r="G113" s="23"/>
+    </row>
+    <row r="114" ht="15.75" customHeight="1">
+      <c r="A114" s="54" t="s">
+        <v>208</v>
+      </c>
+      <c r="B114" s="55" t="s">
+        <v>241</v>
+      </c>
+      <c r="C114" s="56" t="s">
+        <v>242</v>
+      </c>
+      <c r="D114" s="22"/>
+      <c r="E114" s="23"/>
+      <c r="F114" s="57" t="s">
+        <v>243</v>
+      </c>
+      <c r="G114" s="23"/>
+    </row>
+    <row r="115" ht="15.75" customHeight="1">
+      <c r="A115" s="58"/>
+      <c r="B115" s="72"/>
+      <c r="C115" s="73"/>
+      <c r="D115" s="73"/>
+      <c r="E115" s="73"/>
+      <c r="F115" s="74"/>
+      <c r="G115" s="74"/>
+    </row>
     <row r="116" ht="15.75" customHeight="1">
-      <c r="A116" s="1" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="117" ht="15.75" customHeight="1"/>
-    <row r="118" ht="15.75" customHeight="1"/>
+      <c r="A116" s="51" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="117" ht="15.75" customHeight="1">
+      <c r="A117" s="52" t="s">
+        <v>204</v>
+      </c>
+      <c r="B117" s="52" t="s">
+        <v>205</v>
+      </c>
+      <c r="C117" s="53" t="s">
+        <v>206</v>
+      </c>
+      <c r="D117" s="22"/>
+      <c r="E117" s="23"/>
+      <c r="F117" s="53" t="s">
+        <v>207</v>
+      </c>
+      <c r="G117" s="23"/>
+    </row>
+    <row r="118" ht="15.75" customHeight="1">
+      <c r="A118" s="54" t="s">
+        <v>208</v>
+      </c>
+      <c r="B118" s="55" t="s">
+        <v>245</v>
+      </c>
+      <c r="C118" s="56" t="s">
+        <v>246</v>
+      </c>
+      <c r="D118" s="22"/>
+      <c r="E118" s="23"/>
+      <c r="F118" s="57" t="s">
+        <v>247</v>
+      </c>
+      <c r="G118" s="23"/>
+    </row>
     <row r="119" ht="15.75" customHeight="1"/>
     <row r="120" ht="15.75" customHeight="1"/>
-    <row r="121" ht="15.75" customHeight="1"/>
-    <row r="122" ht="15.75" customHeight="1"/>
-    <row r="123" ht="15.75" customHeight="1"/>
-    <row r="124" ht="15.75" customHeight="1"/>
+    <row r="121" ht="15.75" customHeight="1">
+      <c r="A121" s="75" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="122" ht="15.75" customHeight="1">
+      <c r="A122" s="52" t="s">
+        <v>204</v>
+      </c>
+      <c r="B122" s="52" t="s">
+        <v>205</v>
+      </c>
+      <c r="C122" s="53" t="s">
+        <v>206</v>
+      </c>
+      <c r="D122" s="22"/>
+      <c r="E122" s="23"/>
+      <c r="F122" s="53" t="s">
+        <v>207</v>
+      </c>
+      <c r="G122" s="23"/>
+    </row>
+    <row r="123" ht="15.75" customHeight="1">
+      <c r="A123" s="54" t="s">
+        <v>208</v>
+      </c>
+      <c r="B123" s="55" t="s">
+        <v>249</v>
+      </c>
+      <c r="C123" s="56" t="s">
+        <v>250</v>
+      </c>
+      <c r="D123" s="22"/>
+      <c r="E123" s="23"/>
+      <c r="F123" s="57" t="s">
+        <v>251</v>
+      </c>
+      <c r="G123" s="23"/>
+    </row>
+    <row r="124" ht="15.75" customHeight="1">
+      <c r="A124" s="54" t="s">
+        <v>216</v>
+      </c>
+      <c r="B124" s="55" t="s">
+        <v>252</v>
+      </c>
+      <c r="C124" s="56" t="s">
+        <v>253</v>
+      </c>
+      <c r="D124" s="22"/>
+      <c r="E124" s="23"/>
+      <c r="F124" s="57" t="s">
+        <v>254</v>
+      </c>
+      <c r="G124" s="23"/>
+    </row>
     <row r="125" ht="15.75" customHeight="1"/>
-    <row r="126" ht="15.75" customHeight="1"/>
-    <row r="127" ht="15.75" customHeight="1"/>
-    <row r="128" ht="15.75" customHeight="1"/>
-    <row r="129" ht="15.75" customHeight="1"/>
-    <row r="130" ht="15.75" customHeight="1"/>
+    <row r="126" ht="15.75" customHeight="1">
+      <c r="A126" s="1"/>
+    </row>
+    <row r="127" ht="15.75" customHeight="1">
+      <c r="A127" s="75" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="128" ht="15.75" customHeight="1">
+      <c r="A128" s="52" t="s">
+        <v>204</v>
+      </c>
+      <c r="B128" s="52" t="s">
+        <v>205</v>
+      </c>
+      <c r="C128" s="53" t="s">
+        <v>206</v>
+      </c>
+      <c r="D128" s="22"/>
+      <c r="E128" s="23"/>
+      <c r="F128" s="53" t="s">
+        <v>207</v>
+      </c>
+      <c r="G128" s="23"/>
+    </row>
+    <row r="129" ht="15.75" customHeight="1">
+      <c r="A129" s="54" t="s">
+        <v>208</v>
+      </c>
+      <c r="B129" s="55" t="s">
+        <v>256</v>
+      </c>
+      <c r="C129" s="56" t="s">
+        <v>257</v>
+      </c>
+      <c r="D129" s="22"/>
+      <c r="E129" s="23"/>
+      <c r="F129" s="57" t="s">
+        <v>258</v>
+      </c>
+      <c r="G129" s="23"/>
+    </row>
+    <row r="130" ht="15.75" customHeight="1">
+      <c r="A130" s="54" t="s">
+        <v>216</v>
+      </c>
+      <c r="B130" s="55" t="s">
+        <v>259</v>
+      </c>
+      <c r="C130" s="56" t="s">
+        <v>260</v>
+      </c>
+      <c r="D130" s="22"/>
+      <c r="E130" s="23"/>
+      <c r="F130" s="57" t="s">
+        <v>197</v>
+      </c>
+      <c r="G130" s="23"/>
+    </row>
     <row r="131" ht="15.75" customHeight="1"/>
     <row r="132" ht="15.75" customHeight="1"/>
     <row r="133" ht="15.75" customHeight="1"/>
@@ -65509,45 +65982,63 @@
     <row r="1068" ht="15.75" customHeight="1"/>
     <row r="1069" ht="15.75" customHeight="1"/>
     <row r="1070" ht="15.75" customHeight="1"/>
+    <row r="1071" ht="15.75" customHeight="1"/>
+    <row r="1072" ht="15.75" customHeight="1"/>
+    <row r="1073" ht="15.75" customHeight="1"/>
+    <row r="1074" ht="15.75" customHeight="1"/>
+    <row r="1075" ht="15.75" customHeight="1"/>
+    <row r="1076" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="37">
-    <mergeCell ref="C93:E93"/>
-    <mergeCell ref="F93:G93"/>
+  <mergeCells count="49">
+    <mergeCell ref="F95:G95"/>
+    <mergeCell ref="F96:G96"/>
+    <mergeCell ref="F97:G97"/>
+    <mergeCell ref="F98:G98"/>
+    <mergeCell ref="F103:G103"/>
+    <mergeCell ref="F104:G104"/>
+    <mergeCell ref="A105:B105"/>
+    <mergeCell ref="F106:G106"/>
+    <mergeCell ref="C98:E98"/>
+    <mergeCell ref="C104:E104"/>
+    <mergeCell ref="C106:E106"/>
+    <mergeCell ref="C103:E103"/>
+    <mergeCell ref="F107:G107"/>
+    <mergeCell ref="A108:B108"/>
+    <mergeCell ref="F109:G109"/>
+    <mergeCell ref="F110:G110"/>
+    <mergeCell ref="C109:E109"/>
+    <mergeCell ref="C110:E110"/>
+    <mergeCell ref="C107:E107"/>
+    <mergeCell ref="F113:G113"/>
+    <mergeCell ref="F114:G114"/>
+    <mergeCell ref="F117:G117"/>
+    <mergeCell ref="C114:E114"/>
+    <mergeCell ref="C113:E113"/>
+    <mergeCell ref="C117:E117"/>
+    <mergeCell ref="C118:E118"/>
+    <mergeCell ref="C95:E95"/>
+    <mergeCell ref="C96:E96"/>
+    <mergeCell ref="C97:E97"/>
+    <mergeCell ref="F89:G89"/>
+    <mergeCell ref="F90:G90"/>
+    <mergeCell ref="F94:G94"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="C79:E79"/>
-    <mergeCell ref="F79:G79"/>
-    <mergeCell ref="C83:E83"/>
-    <mergeCell ref="F83:G83"/>
-    <mergeCell ref="F78:G78"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="C84:E84"/>
-    <mergeCell ref="F84:G84"/>
-    <mergeCell ref="C85:E85"/>
-    <mergeCell ref="F85:G85"/>
-    <mergeCell ref="C86:E86"/>
-    <mergeCell ref="F86:G86"/>
-    <mergeCell ref="F87:G87"/>
-    <mergeCell ref="C87:E87"/>
-    <mergeCell ref="F95:G95"/>
-    <mergeCell ref="C95:E95"/>
-    <mergeCell ref="A94:B94"/>
-    <mergeCell ref="C92:E92"/>
-    <mergeCell ref="F92:G92"/>
-    <mergeCell ref="C103:E103"/>
-    <mergeCell ref="F103:G103"/>
-    <mergeCell ref="C102:E102"/>
-    <mergeCell ref="F102:G102"/>
-    <mergeCell ref="C106:E106"/>
-    <mergeCell ref="F106:G106"/>
-    <mergeCell ref="C107:E107"/>
-    <mergeCell ref="F107:G107"/>
-    <mergeCell ref="C98:E98"/>
-    <mergeCell ref="F98:G98"/>
-    <mergeCell ref="C99:E99"/>
-    <mergeCell ref="F99:G99"/>
-    <mergeCell ref="A97:B97"/>
-    <mergeCell ref="F96:G96"/>
-    <mergeCell ref="C96:E96"/>
+    <mergeCell ref="C90:E90"/>
+    <mergeCell ref="C94:E94"/>
+    <mergeCell ref="C89:E89"/>
+    <mergeCell ref="F123:G123"/>
+    <mergeCell ref="C123:E123"/>
+    <mergeCell ref="C124:E124"/>
+    <mergeCell ref="C122:E122"/>
+    <mergeCell ref="C129:E129"/>
+    <mergeCell ref="C128:E128"/>
+    <mergeCell ref="C130:E130"/>
+    <mergeCell ref="F118:G118"/>
+    <mergeCell ref="F124:G124"/>
+    <mergeCell ref="F122:G122"/>
+    <mergeCell ref="F129:G129"/>
+    <mergeCell ref="F130:G130"/>
+    <mergeCell ref="F128:G128"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.7874015748031497" footer="0.0" header="0.0" left="1.1811023622047243" right="0.7874015748031497" top="0.7874015748031497"/>
@@ -65577,87 +66068,87 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>228</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="76" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="70" t="s">
-        <v>229</v>
-      </c>
-      <c r="C2" s="70" t="s">
-        <v>184</v>
-      </c>
-      <c r="D2" s="70" t="s">
-        <v>230</v>
-      </c>
-      <c r="E2" s="70" t="s">
-        <v>231</v>
-      </c>
-      <c r="F2" s="70" t="s">
-        <v>232</v>
-      </c>
-      <c r="G2" s="70" t="s">
-        <v>233</v>
-      </c>
-      <c r="H2" s="70" t="s">
-        <v>234</v>
-      </c>
-      <c r="I2" s="70" t="s">
-        <v>235</v>
-      </c>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="71"/>
-      <c r="M2" s="71"/>
-      <c r="N2" s="71"/>
-      <c r="O2" s="71"/>
-      <c r="P2" s="71"/>
-      <c r="Q2" s="71"/>
-      <c r="R2" s="71"/>
-      <c r="S2" s="71"/>
-      <c r="T2" s="71"/>
-      <c r="U2" s="71"/>
-      <c r="V2" s="71"/>
-      <c r="W2" s="71"/>
-      <c r="X2" s="71"/>
-      <c r="Y2" s="71"/>
-      <c r="Z2" s="71"/>
+      <c r="B2" s="76" t="s">
+        <v>262</v>
+      </c>
+      <c r="C2" s="76" t="s">
+        <v>206</v>
+      </c>
+      <c r="D2" s="76" t="s">
+        <v>263</v>
+      </c>
+      <c r="E2" s="76" t="s">
+        <v>264</v>
+      </c>
+      <c r="F2" s="76" t="s">
+        <v>265</v>
+      </c>
+      <c r="G2" s="76" t="s">
+        <v>266</v>
+      </c>
+      <c r="H2" s="76" t="s">
+        <v>267</v>
+      </c>
+      <c r="I2" s="76" t="s">
+        <v>268</v>
+      </c>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
+      <c r="L2" s="77"/>
+      <c r="M2" s="77"/>
+      <c r="N2" s="77"/>
+      <c r="O2" s="77"/>
+      <c r="P2" s="77"/>
+      <c r="Q2" s="77"/>
+      <c r="R2" s="77"/>
+      <c r="S2" s="77"/>
+      <c r="T2" s="77"/>
+      <c r="U2" s="77"/>
+      <c r="V2" s="77"/>
+      <c r="W2" s="77"/>
+      <c r="X2" s="77"/>
+      <c r="Y2" s="77"/>
+      <c r="Z2" s="77"/>
     </row>
     <row r="3">
-      <c r="A3" s="72" t="s">
+      <c r="A3" s="78" t="s">
         <v>43</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>236</v>
+        <v>269</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>237</v>
+        <v>270</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="F3" s="73" t="s">
-        <v>239</v>
-      </c>
-      <c r="G3" s="73" t="s">
-        <v>239</v>
-      </c>
-      <c r="H3" s="74" t="s">
-        <v>240</v>
+        <v>271</v>
+      </c>
+      <c r="F3" s="79" t="s">
+        <v>272</v>
+      </c>
+      <c r="G3" s="79" t="s">
+        <v>272</v>
+      </c>
+      <c r="H3" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="J3" s="71"/>
-      <c r="K3" s="71"/>
-      <c r="L3" s="71"/>
-      <c r="M3" s="71"/>
+        <v>274</v>
+      </c>
+      <c r="J3" s="77"/>
+      <c r="K3" s="77"/>
+      <c r="L3" s="77"/>
+      <c r="M3" s="77"/>
       <c r="N3" s="31"/>
       <c r="O3" s="31"/>
       <c r="P3" s="31"/>
@@ -65667,743 +66158,743 @@
       <c r="T3" s="31"/>
       <c r="U3" s="31"/>
       <c r="V3" s="31"/>
-      <c r="W3" s="71"/>
-      <c r="X3" s="71"/>
-      <c r="Y3" s="71"/>
-      <c r="Z3" s="71"/>
+      <c r="W3" s="77"/>
+      <c r="X3" s="77"/>
+      <c r="Y3" s="77"/>
+      <c r="Z3" s="77"/>
     </row>
     <row r="4">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="78" t="s">
         <v>46</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>242</v>
+        <v>275</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>237</v>
+        <v>270</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="F4" s="73" t="s">
-        <v>244</v>
-      </c>
-      <c r="G4" s="73" t="s">
-        <v>244</v>
-      </c>
-      <c r="H4" s="74" t="s">
-        <v>240</v>
+        <v>276</v>
+      </c>
+      <c r="F4" s="79" t="s">
+        <v>277</v>
+      </c>
+      <c r="G4" s="79" t="s">
+        <v>277</v>
+      </c>
+      <c r="H4" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="J4" s="71"/>
-      <c r="K4" s="71"/>
-      <c r="L4" s="71"/>
-      <c r="M4" s="71"/>
-      <c r="W4" s="71"/>
-      <c r="X4" s="71"/>
-      <c r="Y4" s="71"/>
-      <c r="Z4" s="71"/>
+        <v>278</v>
+      </c>
+      <c r="J4" s="77"/>
+      <c r="K4" s="77"/>
+      <c r="L4" s="77"/>
+      <c r="M4" s="77"/>
+      <c r="W4" s="77"/>
+      <c r="X4" s="77"/>
+      <c r="Y4" s="77"/>
+      <c r="Z4" s="77"/>
     </row>
     <row r="5">
-      <c r="A5" s="72" t="s">
+      <c r="A5" s="78" t="s">
         <v>48</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>246</v>
+        <v>279</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>237</v>
+        <v>270</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="F5" s="73" t="s">
-        <v>244</v>
-      </c>
-      <c r="G5" s="73" t="s">
-        <v>244</v>
-      </c>
-      <c r="H5" s="74" t="s">
-        <v>240</v>
+        <v>280</v>
+      </c>
+      <c r="F5" s="79" t="s">
+        <v>277</v>
+      </c>
+      <c r="G5" s="79" t="s">
+        <v>277</v>
+      </c>
+      <c r="H5" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="J5" s="71"/>
-      <c r="K5" s="71"/>
-      <c r="L5" s="71"/>
-      <c r="M5" s="71"/>
-      <c r="W5" s="71"/>
-      <c r="X5" s="71"/>
-      <c r="Y5" s="71"/>
-      <c r="Z5" s="71"/>
+        <v>281</v>
+      </c>
+      <c r="J5" s="77"/>
+      <c r="K5" s="77"/>
+      <c r="L5" s="77"/>
+      <c r="M5" s="77"/>
+      <c r="W5" s="77"/>
+      <c r="X5" s="77"/>
+      <c r="Y5" s="77"/>
+      <c r="Z5" s="77"/>
     </row>
     <row r="6">
-      <c r="A6" s="74" t="s">
+      <c r="A6" s="80" t="s">
         <v>50</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>249</v>
+        <v>282</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>237</v>
+        <v>270</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="F6" s="73" t="s">
-        <v>251</v>
-      </c>
-      <c r="G6" s="73" t="s">
-        <v>251</v>
-      </c>
-      <c r="H6" s="74" t="s">
-        <v>240</v>
+        <v>283</v>
+      </c>
+      <c r="F6" s="79" t="s">
+        <v>284</v>
+      </c>
+      <c r="G6" s="79" t="s">
+        <v>284</v>
+      </c>
+      <c r="H6" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="J6" s="71"/>
-      <c r="K6" s="71"/>
-      <c r="L6" s="71"/>
-      <c r="M6" s="71"/>
-      <c r="W6" s="71"/>
-      <c r="X6" s="71"/>
-      <c r="Y6" s="71"/>
-      <c r="Z6" s="71"/>
+        <v>285</v>
+      </c>
+      <c r="J6" s="77"/>
+      <c r="K6" s="77"/>
+      <c r="L6" s="77"/>
+      <c r="M6" s="77"/>
+      <c r="W6" s="77"/>
+      <c r="X6" s="77"/>
+      <c r="Y6" s="77"/>
+      <c r="Z6" s="77"/>
     </row>
     <row r="7">
-      <c r="A7" s="74" t="s">
+      <c r="A7" s="80" t="s">
         <v>52</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>53</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>253</v>
+        <v>286</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>237</v>
+        <v>270</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="F7" s="73" t="s">
-        <v>255</v>
-      </c>
-      <c r="G7" s="73" t="s">
-        <v>255</v>
-      </c>
-      <c r="H7" s="74" t="s">
-        <v>240</v>
+        <v>287</v>
+      </c>
+      <c r="F7" s="79" t="s">
+        <v>288</v>
+      </c>
+      <c r="G7" s="79" t="s">
+        <v>288</v>
+      </c>
+      <c r="H7" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="J7" s="71"/>
-      <c r="K7" s="71"/>
-      <c r="L7" s="71"/>
-      <c r="M7" s="71"/>
-      <c r="W7" s="71"/>
-      <c r="X7" s="71"/>
-      <c r="Y7" s="71"/>
-      <c r="Z7" s="71"/>
+        <v>289</v>
+      </c>
+      <c r="J7" s="77"/>
+      <c r="K7" s="77"/>
+      <c r="L7" s="77"/>
+      <c r="M7" s="77"/>
+      <c r="W7" s="77"/>
+      <c r="X7" s="77"/>
+      <c r="Y7" s="77"/>
+      <c r="Z7" s="77"/>
     </row>
     <row r="8">
-      <c r="A8" s="74" t="s">
+      <c r="A8" s="80" t="s">
         <v>54</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>55</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>257</v>
+        <v>290</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>258</v>
+        <v>291</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="F8" s="73" t="b">
+        <v>292</v>
+      </c>
+      <c r="F8" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="G8" s="73" t="b">
+      <c r="G8" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="H8" s="74" t="s">
-        <v>240</v>
+      <c r="H8" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="J8" s="71"/>
-      <c r="K8" s="71"/>
-      <c r="L8" s="71"/>
-      <c r="M8" s="71"/>
-      <c r="W8" s="71"/>
-      <c r="X8" s="71"/>
-      <c r="Y8" s="71"/>
-      <c r="Z8" s="71"/>
+        <v>274</v>
+      </c>
+      <c r="J8" s="77"/>
+      <c r="K8" s="77"/>
+      <c r="L8" s="77"/>
+      <c r="M8" s="77"/>
+      <c r="W8" s="77"/>
+      <c r="X8" s="77"/>
+      <c r="Y8" s="77"/>
+      <c r="Z8" s="77"/>
     </row>
     <row r="9">
-      <c r="A9" s="74" t="s">
+      <c r="A9" s="80" t="s">
         <v>56</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>57</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>260</v>
+        <v>293</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>258</v>
+        <v>291</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="F9" s="73" t="b">
+        <v>294</v>
+      </c>
+      <c r="F9" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="G9" s="73" t="b">
+      <c r="G9" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="H9" s="74" t="s">
-        <v>240</v>
+      <c r="H9" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>248</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="74" t="s">
+      <c r="A10" s="80" t="s">
         <v>58</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>59</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>262</v>
+        <v>295</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>258</v>
+        <v>291</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="F10" s="73" t="b">
+        <v>296</v>
+      </c>
+      <c r="F10" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="G10" s="73" t="b">
+      <c r="G10" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="H10" s="74" t="s">
-        <v>240</v>
+      <c r="H10" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>245</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="74" t="s">
+      <c r="A11" s="80" t="s">
         <v>60</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>61</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>264</v>
+        <v>297</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>258</v>
+        <v>291</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="F11" s="73" t="b">
+        <v>298</v>
+      </c>
+      <c r="F11" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="G11" s="73" t="b">
+      <c r="G11" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="H11" s="74" t="s">
-        <v>240</v>
+      <c r="H11" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>266</v>
+        <v>299</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="74" t="s">
+      <c r="A12" s="80" t="s">
         <v>62</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>63</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>267</v>
+        <v>300</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>268</v>
+        <v>301</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="F12" s="73" t="b">
+        <v>302</v>
+      </c>
+      <c r="F12" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="G12" s="73" t="b">
+      <c r="G12" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="H12" s="74" t="s">
-        <v>240</v>
+      <c r="H12" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>270</v>
+        <v>303</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="74" t="s">
+      <c r="A13" s="80" t="s">
         <v>64</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>65</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>271</v>
+        <v>304</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>272</v>
+        <v>305</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="F13" s="79" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" s="79" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" s="80" t="s">
         <v>273</v>
       </c>
-      <c r="F13" s="73" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="73" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" s="74" t="s">
-        <v>240</v>
-      </c>
       <c r="I13" s="1" t="s">
-        <v>241</v>
+        <v>274</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="74" t="s">
+      <c r="A14" s="80" t="s">
         <v>66</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>67</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>274</v>
+        <v>307</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>272</v>
+        <v>305</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="F14" s="73" t="b">
+        <v>308</v>
+      </c>
+      <c r="F14" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="G14" s="73" t="b">
+      <c r="G14" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="H14" s="74" t="s">
-        <v>240</v>
+      <c r="H14" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>266</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="74" t="s">
+      <c r="A15" s="80" t="s">
         <v>68</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>69</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>276</v>
+        <v>309</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>272</v>
+        <v>305</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="F15" s="73" t="b">
+        <v>296</v>
+      </c>
+      <c r="F15" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="G15" s="73" t="b">
+      <c r="G15" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="H15" s="74" t="s">
-        <v>240</v>
+      <c r="H15" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>248</v>
+        <v>281</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="74" t="s">
+      <c r="A16" s="80" t="s">
         <v>70</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>71</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>277</v>
+        <v>310</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="F16" s="79" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" s="79" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" s="80" t="s">
+        <v>273</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F16" s="73" t="b">
-        <v>1</v>
-      </c>
-      <c r="G16" s="73" t="b">
-        <v>1</v>
-      </c>
-      <c r="H16" s="74" t="s">
-        <v>240</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="N16" s="75"/>
+      <c r="N16" s="81"/>
     </row>
     <row r="17">
-      <c r="A17" s="74" t="s">
+      <c r="A17" s="80" t="s">
         <v>72</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>73</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>280</v>
+        <v>313</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>281</v>
+        <v>314</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="F17" s="73" t="b">
+        <v>302</v>
+      </c>
+      <c r="F17" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="G17" s="73" t="b">
+      <c r="G17" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="H17" s="74" t="s">
-        <v>240</v>
+      <c r="H17" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="N17" s="76"/>
+        <v>315</v>
+      </c>
+      <c r="N17" s="82"/>
     </row>
     <row r="18">
-      <c r="A18" s="74" t="s">
+      <c r="A18" s="80" t="s">
         <v>74</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>75</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>283</v>
+        <v>316</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>284</v>
+        <v>317</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="F18" s="73" t="b">
+        <v>318</v>
+      </c>
+      <c r="F18" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="G18" s="73" t="b">
+      <c r="G18" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="H18" s="74" t="s">
-        <v>240</v>
+      <c r="H18" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="N18" s="77"/>
-      <c r="O18" s="77"/>
-      <c r="P18" s="77"/>
-      <c r="Q18" s="77"/>
-      <c r="R18" s="77"/>
-      <c r="S18" s="77"/>
-      <c r="T18" s="77"/>
-      <c r="U18" s="77"/>
-      <c r="V18" s="77"/>
+        <v>319</v>
+      </c>
+      <c r="N18" s="83"/>
+      <c r="O18" s="83"/>
+      <c r="P18" s="83"/>
+      <c r="Q18" s="83"/>
+      <c r="R18" s="83"/>
+      <c r="S18" s="83"/>
+      <c r="T18" s="83"/>
+      <c r="U18" s="83"/>
+      <c r="V18" s="83"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="74" t="s">
+      <c r="A19" s="80" t="s">
         <v>76</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>65</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>287</v>
+        <v>320</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>288</v>
+        <v>321</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="F19" s="73" t="b">
+        <v>322</v>
+      </c>
+      <c r="F19" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="G19" s="73" t="b">
+      <c r="G19" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="H19" s="74" t="s">
-        <v>240</v>
+      <c r="H19" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="N19" s="76"/>
-      <c r="O19" s="76"/>
-      <c r="P19" s="76"/>
-      <c r="Q19" s="76"/>
-      <c r="R19" s="76"/>
-      <c r="S19" s="76"/>
-      <c r="T19" s="76"/>
-      <c r="U19" s="76"/>
-      <c r="V19" s="76"/>
+        <v>323</v>
+      </c>
+      <c r="N19" s="82"/>
+      <c r="O19" s="82"/>
+      <c r="P19" s="82"/>
+      <c r="Q19" s="82"/>
+      <c r="R19" s="82"/>
+      <c r="S19" s="82"/>
+      <c r="T19" s="82"/>
+      <c r="U19" s="82"/>
+      <c r="V19" s="82"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="74" t="s">
+      <c r="A20" s="80" t="s">
         <v>77</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>73</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>291</v>
+        <v>324</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>292</v>
+        <v>325</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="F20" s="73" t="b">
+        <v>326</v>
+      </c>
+      <c r="F20" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="G20" s="73" t="b">
+      <c r="G20" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="H20" s="74" t="s">
-        <v>240</v>
+      <c r="H20" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="N20" s="76"/>
-      <c r="O20" s="76"/>
-      <c r="P20" s="76"/>
-      <c r="Q20" s="76"/>
-      <c r="R20" s="76"/>
-      <c r="S20" s="76"/>
-      <c r="T20" s="76"/>
-      <c r="U20" s="76"/>
-      <c r="V20" s="76"/>
+        <v>327</v>
+      </c>
+      <c r="N20" s="82"/>
+      <c r="O20" s="82"/>
+      <c r="P20" s="82"/>
+      <c r="Q20" s="82"/>
+      <c r="R20" s="82"/>
+      <c r="S20" s="82"/>
+      <c r="T20" s="82"/>
+      <c r="U20" s="82"/>
+      <c r="V20" s="82"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="74" t="s">
+      <c r="A21" s="80" t="s">
         <v>78</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>79</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>295</v>
+        <v>328</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>296</v>
+        <v>329</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="F21" s="73" t="s">
-        <v>298</v>
-      </c>
-      <c r="G21" s="73" t="s">
-        <v>298</v>
-      </c>
-      <c r="H21" s="74" t="s">
-        <v>240</v>
+        <v>330</v>
+      </c>
+      <c r="F21" s="79" t="s">
+        <v>331</v>
+      </c>
+      <c r="G21" s="79" t="s">
+        <v>331</v>
+      </c>
+      <c r="H21" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="N21" s="76"/>
-      <c r="O21" s="76"/>
-      <c r="P21" s="76"/>
-      <c r="Q21" s="76"/>
-      <c r="R21" s="76"/>
-      <c r="S21" s="76"/>
-      <c r="T21" s="76"/>
-      <c r="U21" s="76"/>
-      <c r="V21" s="76"/>
+        <v>332</v>
+      </c>
+      <c r="N21" s="82"/>
+      <c r="O21" s="82"/>
+      <c r="P21" s="82"/>
+      <c r="Q21" s="82"/>
+      <c r="R21" s="82"/>
+      <c r="S21" s="82"/>
+      <c r="T21" s="82"/>
+      <c r="U21" s="82"/>
+      <c r="V21" s="82"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="74" t="s">
+      <c r="A22" s="80" t="s">
         <v>80</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>63</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>300</v>
+        <v>333</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>301</v>
+        <v>334</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="F22" s="73" t="b">
+        <v>326</v>
+      </c>
+      <c r="F22" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="G22" s="73" t="b">
+      <c r="G22" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="H22" s="74" t="s">
-        <v>240</v>
+      <c r="H22" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="N22" s="76"/>
-      <c r="O22" s="76"/>
-      <c r="P22" s="76"/>
-      <c r="Q22" s="76"/>
-      <c r="R22" s="76"/>
-      <c r="S22" s="76"/>
-      <c r="T22" s="76"/>
-      <c r="U22" s="76"/>
-      <c r="V22" s="76"/>
+        <v>303</v>
+      </c>
+      <c r="N22" s="82"/>
+      <c r="O22" s="82"/>
+      <c r="P22" s="82"/>
+      <c r="Q22" s="82"/>
+      <c r="R22" s="82"/>
+      <c r="S22" s="82"/>
+      <c r="T22" s="82"/>
+      <c r="U22" s="82"/>
+      <c r="V22" s="82"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="74" t="s">
+      <c r="A23" s="80" t="s">
         <v>81</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>82</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>302</v>
+        <v>335</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>303</v>
+        <v>336</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="F23" s="73" t="s">
-        <v>305</v>
-      </c>
-      <c r="G23" s="73" t="s">
-        <v>305</v>
-      </c>
-      <c r="H23" s="74" t="s">
-        <v>240</v>
+        <v>337</v>
+      </c>
+      <c r="F23" s="79" t="s">
+        <v>338</v>
+      </c>
+      <c r="G23" s="79" t="s">
+        <v>338</v>
+      </c>
+      <c r="H23" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="N23" s="76"/>
-      <c r="O23" s="76"/>
-      <c r="P23" s="76"/>
-      <c r="Q23" s="76"/>
-      <c r="R23" s="76"/>
-      <c r="S23" s="76"/>
-      <c r="T23" s="76"/>
-      <c r="U23" s="76"/>
-      <c r="V23" s="76"/>
+        <v>274</v>
+      </c>
+      <c r="N23" s="82"/>
+      <c r="O23" s="82"/>
+      <c r="P23" s="82"/>
+      <c r="Q23" s="82"/>
+      <c r="R23" s="82"/>
+      <c r="S23" s="82"/>
+      <c r="T23" s="82"/>
+      <c r="U23" s="82"/>
+      <c r="V23" s="82"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="74" t="s">
+      <c r="A24" s="80" t="s">
         <v>83</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>84</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>306</v>
+        <v>339</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>303</v>
+        <v>336</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="F24" s="73" t="s">
-        <v>244</v>
-      </c>
-      <c r="G24" s="73" t="s">
-        <v>244</v>
-      </c>
-      <c r="H24" s="74" t="s">
-        <v>240</v>
+        <v>340</v>
+      </c>
+      <c r="F24" s="79" t="s">
+        <v>277</v>
+      </c>
+      <c r="G24" s="79" t="s">
+        <v>277</v>
+      </c>
+      <c r="H24" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>248</v>
+        <v>281</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="74" t="s">
+      <c r="A25" s="80" t="s">
         <v>85</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>79</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>308</v>
+        <v>341</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>309</v>
+        <v>342</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="F25" s="73" t="s">
-        <v>298</v>
-      </c>
-      <c r="G25" s="73" t="s">
-        <v>298</v>
-      </c>
-      <c r="H25" s="74" t="s">
-        <v>240</v>
+        <v>337</v>
+      </c>
+      <c r="F25" s="79" t="s">
+        <v>331</v>
+      </c>
+      <c r="G25" s="79" t="s">
+        <v>331</v>
+      </c>
+      <c r="H25" s="80" t="s">
+        <v>273</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>299</v>
+        <v>332</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -66411,28 +66902,28 @@
         <v>86</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>310</v>
+        <v>343</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>311</v>
+        <v>344</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>312</v>
+        <v>345</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="F26" s="73" t="b">
+        <v>346</v>
+      </c>
+      <c r="F26" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="G26" s="73" t="b">
+      <c r="G26" s="79" t="b">
         <v>1</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>314</v>
+        <v>347</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -66440,28 +66931,28 @@
         <v>89</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>315</v>
+        <v>348</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>316</v>
+        <v>349</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>312</v>
+        <v>345</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="F27" s="73" t="b">
+        <v>350</v>
+      </c>
+      <c r="F27" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="G27" s="73" t="b">
+      <c r="G27" s="79" t="b">
         <v>0</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>318</v>
+        <v>351</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
@@ -66469,28 +66960,28 @@
         <v>91</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>319</v>
+        <v>352</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>320</v>
+        <v>353</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>312</v>
+        <v>345</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="F28" s="73" t="b">
+        <v>354</v>
+      </c>
+      <c r="F28" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="G28" s="73" t="b">
+      <c r="G28" s="79" t="b">
         <v>1</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>322</v>
+        <v>355</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
@@ -66498,28 +66989,28 @@
         <v>93</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>323</v>
+        <v>356</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>324</v>
+        <v>357</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>312</v>
+        <v>345</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="F29" s="73" t="b">
+        <v>358</v>
+      </c>
+      <c r="F29" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="G29" s="73" t="b">
+      <c r="G29" s="79" t="b">
         <v>0</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
@@ -66527,28 +67018,28 @@
         <v>95</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>327</v>
+        <v>360</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>328</v>
+        <v>361</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>329</v>
+        <v>362</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>330</v>
-      </c>
-      <c r="F30" s="73" t="b">
+        <v>363</v>
+      </c>
+      <c r="F30" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="G30" s="73" t="b">
+      <c r="G30" s="79" t="b">
         <v>0</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>331</v>
+        <v>364</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
@@ -66556,28 +67047,28 @@
         <v>97</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>332</v>
+        <v>365</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>333</v>
+        <v>366</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>329</v>
+        <v>362</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="F31" s="73" t="b">
+        <v>367</v>
+      </c>
+      <c r="F31" s="79" t="b">
         <v>1</v>
       </c>
-      <c r="G31" s="73" t="b">
+      <c r="G31" s="79" t="b">
         <v>1</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>335</v>
+        <v>368</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
@@ -66585,28 +67076,28 @@
         <v>99</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>336</v>
+        <v>369</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>337</v>
+        <v>370</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>329</v>
+        <v>362</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>338</v>
-      </c>
-      <c r="F32" s="73" t="s">
-        <v>339</v>
-      </c>
-      <c r="G32" s="73" t="b">
+        <v>371</v>
+      </c>
+      <c r="F32" s="79" t="s">
+        <v>372</v>
+      </c>
+      <c r="G32" s="79" t="b">
         <v>0</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>340</v>
+        <v>373</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
@@ -66614,28 +67105,28 @@
         <v>101</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>341</v>
+        <v>374</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>342</v>
+        <v>375</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>329</v>
+        <v>362</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="F33" s="73" t="s">
-        <v>344</v>
-      </c>
-      <c r="G33" s="73" t="b">
+        <v>376</v>
+      </c>
+      <c r="F33" s="79" t="s">
+        <v>377</v>
+      </c>
+      <c r="G33" s="79" t="b">
         <v>1</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>345</v>
+        <v>378</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
@@ -66646,23 +67137,23 @@
         <v>104</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>346</v>
+        <v>379</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>347</v>
+        <v>380</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>348</v>
+        <v>381</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>349</v>
-      </c>
-      <c r="G34" s="78"/>
+        <v>382</v>
+      </c>
+      <c r="G34" s="84"/>
       <c r="H34" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>350</v>
+        <v>383</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
@@ -66673,23 +67164,23 @@
         <v>106</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>351</v>
+        <v>384</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>347</v>
+        <v>380</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>352</v>
+        <v>385</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="G35" s="78"/>
+        <v>386</v>
+      </c>
+      <c r="G35" s="84"/>
       <c r="H35" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>354</v>
+        <v>387</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
@@ -66700,23 +67191,23 @@
         <v>108</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>355</v>
+        <v>388</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>356</v>
+        <v>389</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>357</v>
+        <v>390</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="G36" s="78"/>
+        <v>391</v>
+      </c>
+      <c r="G36" s="84"/>
       <c r="H36" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>359</v>
+        <v>392</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
@@ -66727,23 +67218,23 @@
         <v>110</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>360</v>
+        <v>393</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>356</v>
+        <v>389</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>361</v>
+        <v>394</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>362</v>
-      </c>
-      <c r="G37" s="78"/>
+        <v>395</v>
+      </c>
+      <c r="G37" s="84"/>
       <c r="H37" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>363</v>
+        <v>396</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
@@ -66754,23 +67245,23 @@
         <v>112</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>364</v>
+        <v>397</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>347</v>
+        <v>380</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>365</v>
+        <v>398</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="G38" s="78"/>
+        <v>399</v>
+      </c>
+      <c r="G38" s="84"/>
       <c r="H38" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>367</v>
+        <v>400</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
@@ -66781,23 +67272,23 @@
         <v>114</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>368</v>
+        <v>401</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>347</v>
+        <v>380</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>369</v>
+        <v>402</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="G39" s="78"/>
+        <v>403</v>
+      </c>
+      <c r="G39" s="84"/>
       <c r="H39" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>371</v>
+        <v>404</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
@@ -66808,23 +67299,23 @@
         <v>116</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>372</v>
+        <v>405</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>347</v>
+        <v>380</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>373</v>
+        <v>406</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="G40" s="78"/>
+        <v>407</v>
+      </c>
+      <c r="G40" s="84"/>
       <c r="H40" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>375</v>
+        <v>408</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
@@ -66835,23 +67326,23 @@
         <v>118</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>376</v>
+        <v>409</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>356</v>
+        <v>389</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>377</v>
+        <v>410</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>378</v>
-      </c>
-      <c r="G41" s="78"/>
+        <v>411</v>
+      </c>
+      <c r="G41" s="84"/>
       <c r="H41" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>379</v>
+        <v>412</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
@@ -66862,23 +67353,23 @@
         <v>120</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>380</v>
+        <v>413</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>356</v>
+        <v>389</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>381</v>
+        <v>414</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="G42" s="78"/>
+        <v>415</v>
+      </c>
+      <c r="G42" s="84"/>
       <c r="H42" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>383</v>
+        <v>416</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
@@ -66889,23 +67380,23 @@
         <v>122</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>384</v>
+        <v>417</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>385</v>
+        <v>418</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>386</v>
+        <v>419</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>387</v>
-      </c>
-      <c r="G43" s="78"/>
+        <v>420</v>
+      </c>
+      <c r="G43" s="84"/>
       <c r="H43" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>388</v>
+        <v>421</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
@@ -66916,23 +67407,23 @@
         <v>124</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>389</v>
+        <v>422</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>390</v>
+        <v>423</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>391</v>
+        <v>424</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="G44" s="78"/>
+        <v>425</v>
+      </c>
+      <c r="G44" s="84"/>
       <c r="H44" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>393</v>
+        <v>426</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
@@ -66943,23 +67434,23 @@
         <v>126</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>394</v>
+        <v>427</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>385</v>
+        <v>418</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>395</v>
+        <v>428</v>
       </c>
       <c r="F45" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="G45" s="84"/>
+      <c r="H45" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="I45" s="1" t="s">
         <v>396</v>
-      </c>
-      <c r="G45" s="78"/>
-      <c r="H45" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
@@ -66970,23 +67461,23 @@
         <v>128</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>397</v>
+        <v>430</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>390</v>
+        <v>423</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>398</v>
+        <v>431</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="G46" s="78"/>
+        <v>425</v>
+      </c>
+      <c r="G46" s="84"/>
       <c r="H46" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>399</v>
+        <v>432</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
@@ -66997,23 +67488,23 @@
         <v>130</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>400</v>
+        <v>433</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>385</v>
+        <v>418</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>398</v>
+        <v>431</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G47" s="78"/>
+        <v>434</v>
+      </c>
+      <c r="G47" s="84"/>
       <c r="H47" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>402</v>
+        <v>435</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
@@ -67024,23 +67515,23 @@
         <v>132</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>403</v>
+        <v>436</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>356</v>
+        <v>389</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>404</v>
+        <v>437</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="G48" s="78"/>
+        <v>438</v>
+      </c>
+      <c r="G48" s="84"/>
       <c r="H48" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>406</v>
+        <v>439</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
@@ -67051,23 +67542,23 @@
         <v>134</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>407</v>
+        <v>440</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>356</v>
+        <v>389</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>408</v>
+        <v>441</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>409</v>
-      </c>
-      <c r="G49" s="78"/>
+        <v>442</v>
+      </c>
+      <c r="G49" s="84"/>
       <c r="H49" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>410</v>
+        <v>443</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
@@ -67078,26 +67569,23 @@
         <v>136</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>411</v>
+        <v>444</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>412</v>
+        <v>445</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>413</v>
+        <v>446</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="G50" s="78"/>
+        <v>447</v>
+      </c>
+      <c r="G50" s="84"/>
       <c r="H50" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="O50" s="1" t="s">
-        <v>416</v>
+        <v>448</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
@@ -67108,23 +67596,23 @@
         <v>138</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>417</v>
+        <v>449</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>385</v>
+        <v>418</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>418</v>
+        <v>450</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="G51" s="78"/>
+        <v>451</v>
+      </c>
+      <c r="G51" s="84"/>
       <c r="H51" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>420</v>
+        <v>452</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
@@ -67135,23 +67623,23 @@
         <v>140</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>421</v>
+        <v>453</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>422</v>
+        <v>454</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>423</v>
+        <v>455</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="G52" s="78"/>
+        <v>456</v>
+      </c>
+      <c r="G52" s="84"/>
       <c r="H52" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>425</v>
+        <v>457</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
@@ -67162,23 +67650,23 @@
         <v>142</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>426</v>
+        <v>458</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>427</v>
+        <v>459</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>428</v>
+        <v>460</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>429</v>
-      </c>
-      <c r="G53" s="78"/>
+        <v>461</v>
+      </c>
+      <c r="G53" s="84"/>
       <c r="H53" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>430</v>
+        <v>462</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
@@ -67189,17 +67677,23 @@
         <v>144</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>431</v>
+        <v>463</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>432</v>
+        <v>464</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="F54" s="1"/>
-      <c r="G54" s="1"/>
-      <c r="H54" s="1"/>
+        <v>465</v>
+      </c>
+      <c r="F54" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G54" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>273</v>
+      </c>
       <c r="I54" s="1"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
@@ -67210,17 +67704,23 @@
         <v>146</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>431</v>
+        <v>463</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>432</v>
+        <v>464</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="F55" s="1"/>
-      <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
+        <v>466</v>
+      </c>
+      <c r="F55" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="G55" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>273</v>
+      </c>
       <c r="I55" s="1"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
@@ -67231,17 +67731,23 @@
         <v>148</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>431</v>
+        <v>463</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>432</v>
+        <v>464</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="F56" s="1"/>
-      <c r="G56" s="1"/>
-      <c r="H56" s="1"/>
+        <v>467</v>
+      </c>
+      <c r="F56" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="G56" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>273</v>
+      </c>
       <c r="I56" s="1"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
@@ -67252,503 +67758,785 @@
         <v>150</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>431</v>
+        <v>463</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>432</v>
+        <v>464</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>436</v>
-      </c>
-      <c r="F57" s="1"/>
-      <c r="G57" s="1"/>
-      <c r="H57" s="1"/>
+        <v>468</v>
+      </c>
+      <c r="F57" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="G57" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>273</v>
+      </c>
       <c r="I57" s="1"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="74" t="s">
+      <c r="A58" s="80" t="s">
         <v>151</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>437</v>
+        <v>469</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>438</v>
+        <v>470</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>439</v>
+        <v>471</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>440</v>
+        <v>472</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="G58" s="73" t="b">
+        <v>473</v>
+      </c>
+      <c r="G58" s="79" t="b">
         <v>1</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>331</v>
+        <v>364</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="74" t="s">
+      <c r="A59" s="80" t="s">
         <v>153</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>442</v>
+        <v>474</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>443</v>
+        <v>475</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>439</v>
+        <v>471</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>444</v>
+        <v>476</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="G59" s="73" t="b">
+        <v>477</v>
+      </c>
+      <c r="G59" s="79" t="b">
         <v>0</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>446</v>
+        <v>478</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="74" t="s">
+      <c r="A60" s="80" t="s">
         <v>155</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>447</v>
+        <v>479</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>448</v>
+        <v>480</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>439</v>
+        <v>471</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>449</v>
+        <v>481</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="G60" s="73" t="b">
+        <v>477</v>
+      </c>
+      <c r="G60" s="79" t="b">
         <v>0</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>450</v>
+        <v>482</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="74" t="s">
+      <c r="A61" s="80" t="s">
         <v>157</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>451</v>
+        <v>483</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>452</v>
+        <v>484</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>439</v>
+        <v>471</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>453</v>
+        <v>485</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="G61" s="73" t="b">
+        <v>477</v>
+      </c>
+      <c r="G61" s="79" t="b">
         <v>0</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>450</v>
+        <v>482</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="74" t="s">
+      <c r="A62" s="80" t="s">
         <v>159</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>454</v>
+        <v>486</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>455</v>
+        <v>487</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>439</v>
+        <v>471</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="F62" s="1" t="b">
+        <v>277</v>
+      </c>
+      <c r="F62" s="79" t="b">
         <v>0</v>
       </c>
-      <c r="G62" s="73" t="b">
+      <c r="G62" s="79" t="b">
         <v>0</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>240</v>
+        <v>273</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>456</v>
+        <v>488</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="74" t="s">
+      <c r="A63" s="80" t="s">
         <v>161</v>
       </c>
-      <c r="B63" s="79" t="s">
+      <c r="B63" s="85" t="s">
         <v>162</v>
       </c>
-      <c r="C63" s="79" t="s">
-        <v>457</v>
-      </c>
-      <c r="D63" s="79" t="s">
-        <v>458</v>
-      </c>
-      <c r="E63" s="79" t="s">
-        <v>459</v>
-      </c>
-      <c r="F63" s="79" t="s">
-        <v>460</v>
-      </c>
-      <c r="G63" s="79" t="s">
-        <v>460</v>
-      </c>
-      <c r="H63" s="79" t="s">
-        <v>240</v>
-      </c>
-      <c r="I63" s="79" t="s">
-        <v>331</v>
+      <c r="C63" s="85" t="s">
+        <v>489</v>
+      </c>
+      <c r="D63" s="85" t="s">
+        <v>490</v>
+      </c>
+      <c r="E63" s="85" t="s">
+        <v>491</v>
+      </c>
+      <c r="F63" s="85" t="s">
+        <v>492</v>
+      </c>
+      <c r="G63" s="85" t="s">
+        <v>492</v>
+      </c>
+      <c r="H63" s="85" t="s">
+        <v>273</v>
+      </c>
+      <c r="I63" s="85" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="74" t="s">
+      <c r="A64" s="80" t="s">
         <v>163</v>
       </c>
-      <c r="B64" s="79" t="s">
+      <c r="B64" s="85" t="s">
         <v>164</v>
       </c>
-      <c r="C64" s="79" t="s">
-        <v>461</v>
-      </c>
-      <c r="D64" s="79" t="s">
-        <v>458</v>
-      </c>
-      <c r="E64" s="79" t="s">
-        <v>462</v>
-      </c>
-      <c r="F64" s="79" t="s">
+      <c r="C64" s="85" t="s">
+        <v>493</v>
+      </c>
+      <c r="D64" s="85" t="s">
+        <v>490</v>
+      </c>
+      <c r="E64" s="85" t="s">
+        <v>494</v>
+      </c>
+      <c r="F64" s="85" t="s">
+        <v>495</v>
+      </c>
+      <c r="G64" s="85" t="s">
+        <v>495</v>
+      </c>
+      <c r="H64" s="85" t="s">
+        <v>273</v>
+      </c>
+      <c r="I64" s="85" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="65" ht="15.75" customHeight="1">
+      <c r="A65" s="80" t="s">
+        <v>165</v>
+      </c>
+      <c r="B65" s="85" t="s">
+        <v>166</v>
+      </c>
+      <c r="C65" s="85" t="s">
+        <v>497</v>
+      </c>
+      <c r="D65" s="85" t="s">
+        <v>498</v>
+      </c>
+      <c r="E65" s="85" t="s">
+        <v>499</v>
+      </c>
+      <c r="F65" s="85" t="s">
+        <v>500</v>
+      </c>
+      <c r="G65" s="85" t="s">
+        <v>500</v>
+      </c>
+      <c r="H65" s="85" t="s">
+        <v>273</v>
+      </c>
+      <c r="I65" s="85" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="66" ht="15.75" customHeight="1">
+      <c r="A66" s="80" t="s">
+        <v>167</v>
+      </c>
+      <c r="B66" s="85" t="s">
+        <v>168</v>
+      </c>
+      <c r="C66" s="85" t="s">
+        <v>502</v>
+      </c>
+      <c r="D66" s="85" t="s">
+        <v>503</v>
+      </c>
+      <c r="E66" s="85" t="s">
+        <v>504</v>
+      </c>
+      <c r="F66" s="85" t="s">
+        <v>505</v>
+      </c>
+      <c r="G66" s="85" t="s">
+        <v>505</v>
+      </c>
+      <c r="H66" s="85" t="s">
+        <v>273</v>
+      </c>
+      <c r="I66" s="85" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="67" ht="15.75" customHeight="1">
+      <c r="A67" s="80" t="s">
+        <v>169</v>
+      </c>
+      <c r="B67" s="85" t="s">
+        <v>170</v>
+      </c>
+      <c r="C67" s="85" t="s">
+        <v>507</v>
+      </c>
+      <c r="D67" s="85" t="s">
+        <v>508</v>
+      </c>
+      <c r="E67" s="85" t="s">
+        <v>509</v>
+      </c>
+      <c r="F67" s="85" t="s">
+        <v>510</v>
+      </c>
+      <c r="G67" s="85" t="s">
+        <v>510</v>
+      </c>
+      <c r="H67" s="85" t="s">
+        <v>273</v>
+      </c>
+      <c r="I67" s="85" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="68" ht="15.75" customHeight="1">
+      <c r="A68" s="80" t="s">
+        <v>171</v>
+      </c>
+      <c r="B68" s="85" t="s">
+        <v>172</v>
+      </c>
+      <c r="C68" s="85" t="s">
+        <v>511</v>
+      </c>
+      <c r="D68" s="85" t="s">
+        <v>508</v>
+      </c>
+      <c r="E68" s="85" t="s">
+        <v>512</v>
+      </c>
+      <c r="F68" s="85" t="s">
+        <v>513</v>
+      </c>
+      <c r="G68" s="85" t="s">
+        <v>513</v>
+      </c>
+      <c r="H68" s="85" t="s">
+        <v>273</v>
+      </c>
+      <c r="I68" s="85" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="69" ht="15.75" customHeight="1">
+      <c r="A69" s="80" t="s">
+        <v>173</v>
+      </c>
+      <c r="B69" s="85" t="s">
+        <v>174</v>
+      </c>
+      <c r="C69" s="85" t="s">
+        <v>515</v>
+      </c>
+      <c r="D69" s="85" t="s">
+        <v>516</v>
+      </c>
+      <c r="E69" s="85" t="s">
+        <v>517</v>
+      </c>
+      <c r="F69" s="85" t="s">
+        <v>518</v>
+      </c>
+      <c r="G69" s="85" t="s">
+        <v>518</v>
+      </c>
+      <c r="H69" s="85" t="s">
+        <v>273</v>
+      </c>
+      <c r="I69" s="85" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="70" ht="15.75" customHeight="1">
+      <c r="A70" s="80" t="s">
+        <v>175</v>
+      </c>
+      <c r="B70" s="85" t="s">
+        <v>176</v>
+      </c>
+      <c r="C70" s="85" t="s">
+        <v>520</v>
+      </c>
+      <c r="D70" s="85" t="s">
+        <v>521</v>
+      </c>
+      <c r="E70" s="85" t="s">
+        <v>522</v>
+      </c>
+      <c r="F70" s="85" t="s">
+        <v>523</v>
+      </c>
+      <c r="G70" s="85" t="s">
+        <v>523</v>
+      </c>
+      <c r="H70" s="85" t="s">
+        <v>273</v>
+      </c>
+      <c r="I70" s="85" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="71" ht="15.75" customHeight="1">
+      <c r="A71" s="80" t="s">
+        <v>177</v>
+      </c>
+      <c r="B71" s="85" t="s">
+        <v>178</v>
+      </c>
+      <c r="C71" s="85" t="s">
+        <v>525</v>
+      </c>
+      <c r="D71" s="85" t="s">
+        <v>526</v>
+      </c>
+      <c r="E71" s="85" t="s">
+        <v>527</v>
+      </c>
+      <c r="F71" s="85" t="s">
+        <v>528</v>
+      </c>
+      <c r="G71" s="85" t="s">
+        <v>528</v>
+      </c>
+      <c r="H71" s="85" t="s">
+        <v>273</v>
+      </c>
+      <c r="I71" s="85" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="72" ht="15.75" customHeight="1">
+      <c r="A72" s="80" t="s">
+        <v>179</v>
+      </c>
+      <c r="B72" s="85" t="s">
+        <v>180</v>
+      </c>
+      <c r="C72" s="85" t="s">
+        <v>530</v>
+      </c>
+      <c r="D72" s="85" t="s">
+        <v>531</v>
+      </c>
+      <c r="E72" s="85" t="s">
+        <v>532</v>
+      </c>
+      <c r="F72" s="85" t="s">
+        <v>533</v>
+      </c>
+      <c r="G72" s="85" t="s">
+        <v>533</v>
+      </c>
+      <c r="H72" s="85" t="s">
+        <v>273</v>
+      </c>
+      <c r="I72" s="85" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="73" ht="15.75" customHeight="1">
+      <c r="A73" s="80" t="s">
+        <v>181</v>
+      </c>
+      <c r="B73" s="86" t="s">
+        <v>182</v>
+      </c>
+      <c r="C73" s="86" t="s">
         <v>463</v>
       </c>
-      <c r="G64" s="79" t="s">
+      <c r="D73" s="86" t="s">
+        <v>464</v>
+      </c>
+      <c r="E73" s="86" t="s">
+        <v>535</v>
+      </c>
+      <c r="F73" s="86">
+        <v>5.0</v>
+      </c>
+      <c r="G73" s="86">
+        <v>5.0</v>
+      </c>
+      <c r="H73" s="86" t="s">
+        <v>273</v>
+      </c>
+      <c r="I73" s="85"/>
+    </row>
+    <row r="74" ht="15.75" customHeight="1">
+      <c r="A74" s="80" t="s">
+        <v>183</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C74" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="H64" s="79" t="s">
-        <v>240</v>
-      </c>
-      <c r="I64" s="79" t="s">
+      <c r="D74" s="1" t="s">
         <v>464</v>
       </c>
-    </row>
-    <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="74" t="s">
-        <v>165</v>
-      </c>
-      <c r="B65" s="79" t="s">
-        <v>166</v>
-      </c>
-      <c r="C65" s="79" t="s">
-        <v>465</v>
-      </c>
-      <c r="D65" s="79" t="s">
-        <v>466</v>
-      </c>
-      <c r="E65" s="79" t="s">
-        <v>467</v>
-      </c>
-      <c r="F65" s="79" t="s">
-        <v>468</v>
-      </c>
-      <c r="G65" s="79" t="s">
-        <v>468</v>
-      </c>
-      <c r="H65" s="79" t="s">
-        <v>240</v>
-      </c>
-      <c r="I65" s="79" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="74" t="s">
-        <v>167</v>
-      </c>
-      <c r="B66" s="79" t="s">
-        <v>168</v>
-      </c>
-      <c r="C66" s="79" t="s">
-        <v>470</v>
-      </c>
-      <c r="D66" s="79" t="s">
-        <v>471</v>
-      </c>
-      <c r="E66" s="79" t="s">
-        <v>472</v>
-      </c>
-      <c r="F66" s="79" t="s">
-        <v>473</v>
-      </c>
-      <c r="G66" s="79" t="s">
-        <v>473</v>
-      </c>
-      <c r="H66" s="79" t="s">
-        <v>240</v>
-      </c>
-      <c r="I66" s="79" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="74" t="s">
-        <v>169</v>
-      </c>
-      <c r="B67" s="79" t="s">
-        <v>170</v>
-      </c>
-      <c r="C67" s="79" t="s">
-        <v>475</v>
-      </c>
-      <c r="D67" s="79" t="s">
-        <v>476</v>
-      </c>
-      <c r="E67" s="79" t="s">
-        <v>477</v>
-      </c>
-      <c r="F67" s="79" t="s">
-        <v>478</v>
-      </c>
-      <c r="G67" s="79" t="s">
-        <v>478</v>
-      </c>
-      <c r="H67" s="79" t="s">
-        <v>240</v>
-      </c>
-      <c r="I67" s="79" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="74" t="s">
-        <v>171</v>
-      </c>
-      <c r="B68" s="79" t="s">
-        <v>172</v>
-      </c>
-      <c r="C68" s="79" t="s">
-        <v>479</v>
-      </c>
-      <c r="D68" s="79" t="s">
-        <v>476</v>
-      </c>
-      <c r="E68" s="79" t="s">
-        <v>480</v>
-      </c>
-      <c r="F68" s="79" t="s">
-        <v>481</v>
-      </c>
-      <c r="G68" s="79" t="s">
-        <v>481</v>
-      </c>
-      <c r="H68" s="79" t="s">
-        <v>240</v>
-      </c>
-      <c r="I68" s="79" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="74" t="s">
-        <v>173</v>
-      </c>
-      <c r="B69" s="79" t="s">
-        <v>174</v>
-      </c>
-      <c r="C69" s="79" t="s">
-        <v>483</v>
-      </c>
-      <c r="D69" s="79" t="s">
-        <v>484</v>
-      </c>
-      <c r="E69" s="79" t="s">
-        <v>485</v>
-      </c>
-      <c r="F69" s="79" t="s">
-        <v>486</v>
-      </c>
-      <c r="G69" s="79" t="s">
-        <v>486</v>
-      </c>
-      <c r="H69" s="79" t="s">
-        <v>240</v>
-      </c>
-      <c r="I69" s="79" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="74" t="s">
-        <v>175</v>
-      </c>
-      <c r="B70" s="79" t="s">
-        <v>176</v>
-      </c>
-      <c r="C70" s="79" t="s">
-        <v>488</v>
-      </c>
-      <c r="D70" s="79" t="s">
-        <v>489</v>
-      </c>
-      <c r="E70" s="79" t="s">
-        <v>490</v>
-      </c>
-      <c r="F70" s="79" t="s">
-        <v>491</v>
-      </c>
-      <c r="G70" s="79" t="s">
-        <v>491</v>
-      </c>
-      <c r="H70" s="79" t="s">
-        <v>240</v>
-      </c>
-      <c r="I70" s="79" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="74" t="s">
-        <v>177</v>
-      </c>
-      <c r="B71" s="79" t="s">
-        <v>178</v>
-      </c>
-      <c r="C71" s="79" t="s">
-        <v>493</v>
-      </c>
-      <c r="D71" s="79" t="s">
-        <v>494</v>
-      </c>
-      <c r="E71" s="79" t="s">
-        <v>495</v>
-      </c>
-      <c r="F71" s="79" t="s">
-        <v>496</v>
-      </c>
-      <c r="G71" s="79" t="s">
-        <v>496</v>
-      </c>
-      <c r="H71" s="79" t="s">
-        <v>240</v>
-      </c>
-      <c r="I71" s="79" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="74" t="s">
-        <v>179</v>
-      </c>
-      <c r="B72" s="79" t="s">
-        <v>180</v>
-      </c>
-      <c r="C72" s="79" t="s">
-        <v>498</v>
-      </c>
-      <c r="D72" s="79" t="s">
-        <v>499</v>
-      </c>
-      <c r="E72" s="79" t="s">
-        <v>500</v>
-      </c>
-      <c r="F72" s="79" t="s">
-        <v>501</v>
-      </c>
-      <c r="G72" s="79" t="s">
-        <v>501</v>
-      </c>
-      <c r="H72" s="79" t="s">
-        <v>240</v>
-      </c>
-      <c r="I72" s="79" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="74"/>
-    </row>
-    <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="79"/>
-      <c r="B74" s="80" t="s">
-        <v>503</v>
-      </c>
-      <c r="C74" s="79"/>
+      <c r="E74" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="F74" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G74" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>273</v>
+      </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="79"/>
-      <c r="B75" s="81" t="s">
-        <v>504</v>
-      </c>
-      <c r="C75" s="79"/>
+      <c r="A75" s="80" t="s">
+        <v>185</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="F75" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="G75" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>273</v>
+      </c>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="79"/>
-      <c r="B76" s="81" t="s">
-        <v>505</v>
-      </c>
-      <c r="C76" s="79"/>
+      <c r="A76" s="80" t="s">
+        <v>187</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="F76" s="1">
+        <v>7.0</v>
+      </c>
+      <c r="G76" s="1">
+        <v>7.0</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>273</v>
+      </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="79"/>
-      <c r="B77" s="81" t="s">
-        <v>506</v>
-      </c>
-      <c r="C77" s="79"/>
+      <c r="A77" s="80" t="s">
+        <v>189</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="F77" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G77" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>273</v>
+      </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="79"/>
-      <c r="B78" s="81" t="s">
-        <v>507</v>
-      </c>
-      <c r="C78" s="79"/>
-    </row>
-    <row r="79" ht="15.75" customHeight="1"/>
-    <row r="80" ht="15.75" customHeight="1"/>
-    <row r="81" ht="15.75" customHeight="1"/>
-    <row r="82" ht="15.75" customHeight="1"/>
-    <row r="83" ht="15.75" customHeight="1"/>
-    <row r="84" ht="15.75" customHeight="1"/>
-    <row r="85" ht="15.75" customHeight="1"/>
-    <row r="86" ht="15.75" customHeight="1"/>
-    <row r="87" ht="15.75" customHeight="1"/>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1"/>
+      <c r="A78" s="80" t="s">
+        <v>191</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="F78" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="G78" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="79" ht="15.75" customHeight="1">
+      <c r="A79" s="80" t="s">
+        <v>193</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="F79" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="G79" s="1">
+        <v>0.0</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="80" ht="15.75" customHeight="1">
+      <c r="A80" s="80" t="s">
+        <v>195</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="E80" s="87" t="s">
+        <v>543</v>
+      </c>
+      <c r="F80" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="G80" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="81" ht="15.75" customHeight="1">
+      <c r="A81" s="80" t="s">
+        <v>197</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="82" ht="15.75" customHeight="1">
+      <c r="A82" s="80" t="s">
+        <v>199</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="F82" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="G82" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="83" ht="15.75" customHeight="1">
+      <c r="A83" s="80" t="s">
+        <v>201</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="F83" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="G83" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="84" ht="15.75" customHeight="1">
+      <c r="A84" s="80"/>
+    </row>
+    <row r="85" ht="15.75" customHeight="1">
+      <c r="A85" s="85"/>
+      <c r="B85" s="88" t="s">
+        <v>552</v>
+      </c>
+      <c r="C85" s="85"/>
+    </row>
+    <row r="86" ht="15.75" customHeight="1">
+      <c r="A86" s="85"/>
+      <c r="B86" s="89" t="s">
+        <v>553</v>
+      </c>
+      <c r="C86" s="85"/>
+    </row>
+    <row r="87" ht="15.75" customHeight="1">
+      <c r="A87" s="85"/>
+      <c r="B87" s="89" t="s">
+        <v>554</v>
+      </c>
+      <c r="C87" s="85"/>
+    </row>
+    <row r="88" ht="15.75" customHeight="1">
+      <c r="A88" s="85"/>
+      <c r="B88" s="89" t="s">
+        <v>555</v>
+      </c>
+      <c r="C88" s="85"/>
+    </row>
+    <row r="89" ht="15.75" customHeight="1">
+      <c r="A89" s="85"/>
+      <c r="B89" s="89" t="s">
+        <v>556</v>
+      </c>
+      <c r="C89" s="85"/>
+    </row>
     <row r="90" ht="15.75" customHeight="1"/>
     <row r="91" ht="15.75" customHeight="1"/>
     <row r="92" ht="15.75" customHeight="1"/>
@@ -68704,10 +69492,24 @@
     <row r="1042" ht="15.75" customHeight="1"/>
     <row r="1043" ht="15.75" customHeight="1"/>
     <row r="1044" ht="15.75" customHeight="1"/>
+    <row r="1045" ht="15.75" customHeight="1"/>
+    <row r="1046" ht="15.75" customHeight="1"/>
+    <row r="1047" ht="15.75" customHeight="1"/>
+    <row r="1048" ht="15.75" customHeight="1"/>
+    <row r="1049" ht="15.75" customHeight="1"/>
+    <row r="1050" ht="15.75" customHeight="1"/>
+    <row r="1051" ht="15.75" customHeight="1"/>
+    <row r="1052" ht="15.75" customHeight="1"/>
+    <row r="1053" ht="15.75" customHeight="1"/>
+    <row r="1054" ht="15.75" customHeight="1"/>
+    <row r="1055" ht="15.75" customHeight="1"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="E80"/>
+  </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.7874015748031497" footer="0.0" header="0.0" left="1.1811023622047245" right="0.7874015748031497" top="0.7874015748031497"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>